<commit_message>
Update Smart Attendance System
</commit_message>
<xml_diff>
--- a/class_activity.xlsx
+++ b/class_activity.xlsx
@@ -481,7 +481,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>semester1</t>
+          <t>SEMESTER1</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -498,12 +498,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Khan sir</t>
+          <t>Menal Ma'aM</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -512,32 +512,32 @@
         </is>
       </c>
       <c r="G2" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>46</v>
+        <v>0</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>65.71%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>Fail</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>semester1</t>
+          <t>SEMESTER1</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -554,46 +554,46 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Khan sir</t>
+          <t>Menal Ma'aM</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>DBMS</t>
+          <t>HTML</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="I3" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>55</v>
+        <v>0</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>78.57%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Very Good</t>
+          <t>Fail</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>semester1</t>
+          <t>SEMESTER1</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -610,46 +610,46 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Khan sir</t>
+          <t>Menal Ma'aM</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>HTML</t>
+          <t>DBMS</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="I4" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>51</v>
+        <v>0</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>72.86%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>Fail</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>semester1</t>
+          <t>SEMESTER1</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -666,12 +666,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Khan sir</t>
+          <t>Menal Ma'aM</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -680,32 +680,32 @@
         </is>
       </c>
       <c r="G5" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>62</v>
+        <v>0</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>88.57%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Very Good</t>
+          <t>Fail</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>semester1</t>
+          <t>SEMESTER1</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -722,46 +722,46 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Khan sir</t>
+          <t>Menal Ma'aM</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>DBMS</t>
+          <t>HTML</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="I6" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="J6" t="n">
-        <v>59</v>
+        <v>0</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>84.29%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>Very Good</t>
+          <t>Fail</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>semester1</t>
+          <t>SEMESTER1</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -778,46 +778,46 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Khan sir</t>
+          <t>Menal Ma'aM</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>HTML</t>
+          <t>DBMS</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>55</v>
+        <v>0</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>78.57%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>Very Good</t>
+          <t>Fail</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>semester1</t>
+          <t>SEMESTER1</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -834,12 +834,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Khan sir</t>
+          <t>Menal Ma'aM</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -848,32 +848,32 @@
         </is>
       </c>
       <c r="G8" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="I8" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>48</v>
+        <v>0</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>68.57%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>Fail</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>semester1</t>
+          <t>SEMESTER1</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -890,46 +890,46 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Khan sir</t>
+          <t>Menal Ma'aM</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>DBMS</t>
+          <t>HTML</t>
         </is>
       </c>
       <c r="G9" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="I9" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>53</v>
+        <v>0</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>75.71%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Very Good</t>
+          <t>Fail</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>semester1</t>
+          <t>SEMESTER1</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -946,39 +946,39 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Khan sir</t>
+          <t>Menal Ma'aM</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>HTML</t>
+          <t>DBMS</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>58</v>
+        <v>0</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>82.86%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Very Good</t>
+          <t>Fail</t>
         </is>
       </c>
     </row>

</xml_diff>